<commit_message>
Adiciona analises de consumo e crescimento por item
</commit_message>
<xml_diff>
--- a/data-source/COMPRATRANSFER.xlsx
+++ b/data-source/COMPRATRANSFER.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5b319cc1648f3add/Área de Trabalho/TRANSFER-ANALISE/data-source/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="81" documentId="8_{77FF3A89-80B9-407D-BABF-BDBB720C2313}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5768AC1C-723C-4607-B6EB-C72EC8542A72}"/>
+  <xr:revisionPtr revIDLastSave="133" documentId="8_{77FF3A89-80B9-407D-BABF-BDBB720C2313}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5530CB9A-AC36-4CC2-92DD-6069CA72705B}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,6 +16,7 @@
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Plan1!$A$1:$I$22</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">Plan1!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="24">
   <si>
     <t>Núm.OC</t>
   </si>
@@ -62,9 +63,6 @@
     <t>TRANSFER TOTAL METALIC FILM SILVER QT-001A - AMERICA ASIA</t>
   </si>
   <si>
-    <t>TRANSFER TOTAL METALIC FILM GRAFITE QT-339A - AMERICA ASIA</t>
-  </si>
-  <si>
     <t>DOTS FILM LASER - AMERICA ASIA</t>
   </si>
   <si>
@@ -105,6 +103,12 @@
   </si>
   <si>
     <t>PROTECTION FILM 35UM - AMERICA ASIA</t>
+  </si>
+  <si>
+    <t>28/0/2026</t>
+  </si>
+  <si>
+    <t>TRANSFER TOTAL METALIC FILM PEWTER QT-110A - AMERICA ASIA</t>
   </si>
 </sst>
 </file>
@@ -130,7 +134,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -140,12 +144,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC0C0C0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -187,14 +185,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -565,18 +566,18 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H1" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I1" s="5" t="s">
         <v>15</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="3">
-        <v>1255</v>
+        <v>1467</v>
       </c>
       <c r="B2" s="3">
         <v>162</v>
@@ -585,27 +586,27 @@
         <v>6</v>
       </c>
       <c r="D2" s="4">
-        <v>46156</v>
+        <v>46204</v>
       </c>
       <c r="E2" s="3">
-        <v>7485</v>
+        <v>4413</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G2" s="6">
-        <v>6000</v>
+        <v>8</v>
+      </c>
+      <c r="G2" s="7">
+        <v>3000</v>
       </c>
       <c r="H2">
         <v>12</v>
       </c>
       <c r="I2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
-        <v>1350</v>
+        <v>1469</v>
       </c>
       <c r="B3" s="3">
         <v>162</v>
@@ -614,27 +615,27 @@
         <v>6</v>
       </c>
       <c r="D3" s="4">
-        <v>46176</v>
+        <v>46204</v>
       </c>
       <c r="E3" s="3">
-        <v>7425</v>
+        <v>10090</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G3" s="6">
-        <v>3330</v>
+        <v>10</v>
+      </c>
+      <c r="G3" s="7">
+        <v>3250</v>
       </c>
       <c r="H3">
         <v>12</v>
       </c>
       <c r="I3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
-        <v>1467</v>
+        <v>1470</v>
       </c>
       <c r="B4" s="3">
         <v>162</v>
@@ -646,24 +647,24 @@
         <v>46204</v>
       </c>
       <c r="E4" s="3">
-        <v>4413</v>
+        <v>12515</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G4" s="6">
-        <v>3000</v>
+        <v>11</v>
+      </c>
+      <c r="G4" s="7">
+        <v>6480</v>
       </c>
       <c r="H4">
         <v>12</v>
       </c>
       <c r="I4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
-        <v>1468</v>
+        <v>1487</v>
       </c>
       <c r="B5" s="3">
         <v>162</v>
@@ -672,27 +673,27 @@
         <v>6</v>
       </c>
       <c r="D5" s="4">
-        <v>46204</v>
+        <v>46206</v>
       </c>
       <c r="E5" s="3">
-        <v>7484</v>
+        <v>17075</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G5" s="6">
-        <v>10620</v>
+        <v>12</v>
+      </c>
+      <c r="G5" s="7">
+        <v>4230</v>
       </c>
       <c r="H5">
         <v>12</v>
       </c>
       <c r="I5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
-        <v>1469</v>
+        <v>1565</v>
       </c>
       <c r="B6" s="3">
         <v>162</v>
@@ -701,27 +702,27 @@
         <v>6</v>
       </c>
       <c r="D6" s="4">
-        <v>46204</v>
+        <v>46225</v>
       </c>
       <c r="E6" s="3">
-        <v>10090</v>
+        <v>7484</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G6" s="6">
-        <v>3000</v>
+        <v>9</v>
+      </c>
+      <c r="G6" s="7">
+        <v>9000</v>
       </c>
       <c r="H6">
         <v>12</v>
       </c>
       <c r="I6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
-        <v>1470</v>
+        <v>1565</v>
       </c>
       <c r="B7" s="3">
         <v>162</v>
@@ -730,27 +731,27 @@
         <v>6</v>
       </c>
       <c r="D7" s="4">
-        <v>46204</v>
+        <v>46225</v>
       </c>
       <c r="E7" s="3">
-        <v>12515</v>
+        <v>7485</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G7" s="6">
+        <v>7</v>
+      </c>
+      <c r="G7" s="7">
         <v>6000</v>
       </c>
       <c r="H7">
         <v>12</v>
       </c>
       <c r="I7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="3">
-        <v>1487</v>
+        <v>1565</v>
       </c>
       <c r="B8" s="3">
         <v>162</v>
@@ -759,22 +760,22 @@
         <v>6</v>
       </c>
       <c r="D8" s="4">
-        <v>46206</v>
+        <v>46225</v>
       </c>
       <c r="E8" s="3">
-        <v>17075</v>
+        <v>10090</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G8" s="6">
-        <v>4000</v>
+        <v>10</v>
+      </c>
+      <c r="G8" s="7">
+        <v>3200</v>
       </c>
       <c r="H8">
         <v>12</v>
       </c>
       <c r="I8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
@@ -791,24 +792,24 @@
         <v>46225</v>
       </c>
       <c r="E9" s="3">
-        <v>7484</v>
+        <v>17076</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G9" s="6">
-        <v>9000</v>
+        <v>13</v>
+      </c>
+      <c r="G9" s="7">
+        <v>3070</v>
       </c>
       <c r="H9">
         <v>12</v>
       </c>
       <c r="I9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="3">
-        <v>1565</v>
+        <v>1582</v>
       </c>
       <c r="B10" s="3">
         <v>162</v>
@@ -817,27 +818,27 @@
         <v>6</v>
       </c>
       <c r="D10" s="4">
-        <v>46225</v>
+        <v>46233</v>
       </c>
       <c r="E10" s="3">
-        <v>7485</v>
+        <v>7484</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G10" s="6">
-        <v>6000</v>
+        <v>9</v>
+      </c>
+      <c r="G10" s="7">
+        <v>8800</v>
       </c>
       <c r="H10">
         <v>12</v>
       </c>
       <c r="I10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="3">
-        <v>1565</v>
+        <v>1582</v>
       </c>
       <c r="B11" s="3">
         <v>162</v>
@@ -846,27 +847,27 @@
         <v>6</v>
       </c>
       <c r="D11" s="4">
-        <v>46225</v>
+        <v>46233</v>
       </c>
       <c r="E11" s="3">
-        <v>10090</v>
+        <v>7485</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G11" s="6">
+        <v>7</v>
+      </c>
+      <c r="G11" s="7">
         <v>3000</v>
       </c>
       <c r="H11">
         <v>12</v>
       </c>
       <c r="I11" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="3">
-        <v>1565</v>
+        <v>1582</v>
       </c>
       <c r="B12" s="3">
         <v>162</v>
@@ -875,27 +876,27 @@
         <v>6</v>
       </c>
       <c r="D12" s="4">
-        <v>46225</v>
+        <v>46233</v>
       </c>
       <c r="E12" s="3">
-        <v>17076</v>
+        <v>10090</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="G12" s="6">
-        <v>3000</v>
+        <v>10</v>
+      </c>
+      <c r="G12" s="7">
+        <v>3100</v>
       </c>
       <c r="H12">
         <v>12</v>
       </c>
       <c r="I12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="3">
-        <v>1582</v>
+        <v>1602</v>
       </c>
       <c r="B13" s="3">
         <v>162</v>
@@ -904,27 +905,27 @@
         <v>6</v>
       </c>
       <c r="D13" s="4">
-        <v>46233</v>
+        <v>46239</v>
       </c>
       <c r="E13" s="3">
         <v>7484</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G13" s="6">
-        <v>9000</v>
+        <v>9</v>
+      </c>
+      <c r="G13" s="7">
+        <v>10100</v>
       </c>
       <c r="H13">
         <v>12</v>
       </c>
       <c r="I13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="3">
-        <v>1582</v>
+        <v>1633</v>
       </c>
       <c r="B14" s="3">
         <v>162</v>
@@ -933,7 +934,7 @@
         <v>6</v>
       </c>
       <c r="D14" s="4">
-        <v>46233</v>
+        <v>46245</v>
       </c>
       <c r="E14" s="3">
         <v>7485</v>
@@ -941,19 +942,19 @@
       <c r="F14" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G14" s="6">
-        <v>3000</v>
+      <c r="G14" s="7">
+        <v>5000</v>
       </c>
       <c r="H14">
         <v>12</v>
       </c>
       <c r="I14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="3">
-        <v>1582</v>
+        <v>1487</v>
       </c>
       <c r="B15" s="3">
         <v>162</v>
@@ -962,27 +963,27 @@
         <v>6</v>
       </c>
       <c r="D15" s="4">
-        <v>46233</v>
+        <v>46206</v>
       </c>
       <c r="E15" s="3">
-        <v>10090</v>
+        <v>17075</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G15" s="6">
-        <v>3000</v>
+        <v>12</v>
+      </c>
+      <c r="G15" s="7">
+        <v>1340</v>
       </c>
       <c r="H15">
         <v>12</v>
       </c>
       <c r="I15" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" s="3">
-        <v>1602</v>
+        <v>1468</v>
       </c>
       <c r="B16" s="3">
         <v>162</v>
@@ -991,27 +992,27 @@
         <v>6</v>
       </c>
       <c r="D16" s="4">
-        <v>46239</v>
+        <v>46204</v>
       </c>
       <c r="E16" s="3">
         <v>7484</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G16" s="6">
+        <v>9</v>
+      </c>
+      <c r="G16" s="7">
         <v>10000</v>
       </c>
       <c r="H16">
         <v>12</v>
       </c>
       <c r="I16" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" s="3">
-        <v>1633</v>
+        <v>1666</v>
       </c>
       <c r="B17" s="3">
         <v>162</v>
@@ -1020,27 +1021,27 @@
         <v>6</v>
       </c>
       <c r="D17" s="4">
-        <v>46245</v>
+        <v>46252</v>
       </c>
       <c r="E17" s="3">
-        <v>7485</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G17" s="6">
-        <v>5000</v>
+        <v>10090</v>
+      </c>
+      <c r="F17" t="s">
+        <v>10</v>
+      </c>
+      <c r="G17" s="7">
+        <v>3000</v>
       </c>
       <c r="H17">
         <v>12</v>
       </c>
       <c r="I17" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" s="3">
-        <v>1487</v>
+        <v>1665</v>
       </c>
       <c r="B18" s="3">
         <v>162</v>
@@ -1049,27 +1050,27 @@
         <v>6</v>
       </c>
       <c r="D18" s="4">
-        <v>46206</v>
+        <v>46252</v>
       </c>
       <c r="E18" s="3">
-        <v>17075</v>
+        <v>7484</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G18" s="6">
-        <v>1340</v>
+        <v>9</v>
+      </c>
+      <c r="G18" s="7">
+        <v>20000</v>
       </c>
       <c r="H18">
         <v>12</v>
       </c>
       <c r="I18" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" s="3">
-        <v>1468</v>
+        <v>1665</v>
       </c>
       <c r="B19" s="3">
         <v>162</v>
@@ -1078,27 +1079,27 @@
         <v>6</v>
       </c>
       <c r="D19" s="4">
-        <v>46204</v>
+        <v>46252</v>
       </c>
       <c r="E19" s="3">
-        <v>7484</v>
+        <v>4413</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G19" s="6">
-        <v>10000</v>
+        <v>8</v>
+      </c>
+      <c r="G19" s="7">
+        <v>3000</v>
       </c>
       <c r="H19">
         <v>12</v>
       </c>
       <c r="I19" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" s="3">
-        <v>1666</v>
+        <v>1668</v>
       </c>
       <c r="B20" s="3">
         <v>162</v>
@@ -1110,24 +1111,24 @@
         <v>46252</v>
       </c>
       <c r="E20" s="3">
-        <v>10090</v>
-      </c>
-      <c r="F20" t="s">
-        <v>11</v>
-      </c>
-      <c r="G20" s="6">
-        <v>3000</v>
+        <v>30189</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G20" s="7">
+        <v>7000</v>
       </c>
       <c r="H20">
         <v>12</v>
       </c>
       <c r="I20" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" s="3">
-        <v>1665</v>
+        <v>1487</v>
       </c>
       <c r="B21" s="3">
         <v>162</v>
@@ -1136,27 +1137,27 @@
         <v>6</v>
       </c>
       <c r="D21" s="4">
-        <v>46252</v>
+        <v>46261</v>
       </c>
       <c r="E21" s="3">
-        <v>7484</v>
+        <v>17075</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G21" s="6">
-        <v>20000</v>
+        <v>12</v>
+      </c>
+      <c r="G21" s="7">
+        <v>2000</v>
       </c>
       <c r="H21">
         <v>12</v>
       </c>
       <c r="I21" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" s="3">
-        <v>1665</v>
+        <v>1666</v>
       </c>
       <c r="B22" s="3">
         <v>162</v>
@@ -1168,12 +1169,12 @@
         <v>46252</v>
       </c>
       <c r="E22" s="3">
-        <v>4413</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G22" s="6">
+        <v>10090</v>
+      </c>
+      <c r="F22" t="s">
+        <v>10</v>
+      </c>
+      <c r="G22" s="7">
         <v>3000</v>
       </c>
       <c r="H22">
@@ -1185,7 +1186,7 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" s="3">
-        <v>1668</v>
+        <v>1697</v>
       </c>
       <c r="B23" s="3">
         <v>162</v>
@@ -1193,26 +1194,27 @@
       <c r="C23" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D23" s="4">
-        <v>46252</v>
+      <c r="D23" t="s">
+        <v>22</v>
       </c>
       <c r="E23" s="3">
-        <v>30189</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G23" s="6">
-        <v>7000</v>
+        <v>9000</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="G23" s="7">
+        <v>1000</v>
       </c>
       <c r="H23">
         <v>12</v>
       </c>
       <c r="I23" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:I22" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <printOptions gridLines="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" fitToHeight="9999" orientation="landscape"/>

</xml_diff>